<commit_message>
some improvements in the arabic words file
</commit_message>
<xml_diff>
--- a/data/Сажида (русс)/2. Слова.xlsx
+++ b/data/Сажида (русс)/2. Слова.xlsx
@@ -27,9 +27,6 @@
     <t>فِي</t>
   </si>
   <si>
-    <t>В, На, К</t>
-  </si>
-  <si>
     <t>أَينَ أَنْتَ؟</t>
   </si>
   <si>
@@ -106,6 +103,9 @@
   </si>
   <si>
     <t>طَالِبٌ</t>
+  </si>
+  <si>
+    <t>В, На, К (предлог)</t>
   </si>
 </sst>
 </file>
@@ -472,10 +472,10 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>5</v>
       </c>
       <c r="K2" s="1"/>
     </row>
@@ -484,114 +484,114 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="C3" s="1"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>7</v>
       </c>
       <c r="C4" s="1"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="C5" s="1"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>11</v>
       </c>
       <c r="C6" s="1"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>15</v>
       </c>
       <c r="C8" s="1"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="C9" s="1"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="C10" s="1"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="C11" s="1"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="C12" s="1"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>25</v>
       </c>
       <c r="C13" s="1"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C14" s="1"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>